<commit_message>
a temporary sparw hero for player 0625-8.56
</commit_message>
<xml_diff>
--- a/Docs/平衡测算文档.xlsx
+++ b/Docs/平衡测算文档.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Warhummer III AdamWorkshop\MyMods\商队Rogue玩法Mod\TotalWarIIIMod-RogueTheWarHammer\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2456B655-3896-491E-AC1E-97E86E20C70C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C634C750-5060-4637-9E3A-432E42FEEA01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="537" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-732" yWindow="4476" windowWidth="30720" windowHeight="14160" tabRatio="537" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1392,7 +1392,7 @@
         <v>2500</v>
       </c>
       <c r="I2" s="1">
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="J2" s="1">
         <v>450</v>
@@ -1485,7 +1485,7 @@
         <v>900</v>
       </c>
       <c r="E5" s="1">
-        <v>1250</v>
+        <v>1200</v>
       </c>
       <c r="F5" s="1">
         <v>1500</v>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="D10" s="1">
         <f>I2</f>
-        <v>4500</v>
+        <v>4000</v>
       </c>
       <c r="E10" s="4"/>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D11" s="1">
         <f>D10+J$2</f>
-        <v>4950</v>
+        <v>4450</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="D12" s="1">
         <f t="shared" ref="D12:D14" si="3">D11+J$2</f>
-        <v>5400</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="D13" s="1">
         <f t="shared" si="3"/>
-        <v>5850</v>
+        <v>5350</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
@@ -1597,11 +1597,11 @@
       </c>
       <c r="D14" s="1">
         <f t="shared" si="3"/>
-        <v>6300</v>
+        <v>5800</v>
       </c>
       <c r="E14" s="1">
         <f>D14*1.25</f>
-        <v>7875</v>
+        <v>7250</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.25">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="D15" s="1">
         <f>D14+K$2</f>
-        <v>7150</v>
+        <v>6650</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.25">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="D16" s="1">
         <f t="shared" ref="D16:D19" si="5">D15+K$2</f>
-        <v>8000</v>
+        <v>7500</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D17" s="1">
         <f t="shared" si="5"/>
-        <v>8850</v>
+        <v>8350</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="D18" s="1">
         <f t="shared" si="5"/>
-        <v>9700</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1686,11 +1686,11 @@
       </c>
       <c r="D19" s="1">
         <f t="shared" si="5"/>
-        <v>10550</v>
+        <v>10050</v>
       </c>
       <c r="E19" s="1">
         <f>D19*1.25</f>
-        <v>13187.5</v>
+        <v>12562.5</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="D20" s="1">
         <f>D19+L$2</f>
-        <v>11500</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="D21" s="1">
         <f t="shared" ref="D21:D24" si="7">D20+L$2</f>
-        <v>12450</v>
+        <v>11950</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="D22" s="1">
         <f t="shared" si="7"/>
-        <v>13400</v>
+        <v>12900</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1758,7 +1758,7 @@
       </c>
       <c r="D23" s="1">
         <f t="shared" si="7"/>
-        <v>14350</v>
+        <v>13850</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1775,11 +1775,11 @@
       </c>
       <c r="D24" s="1">
         <f t="shared" si="7"/>
-        <v>15300</v>
+        <v>14800</v>
       </c>
       <c r="E24" s="1">
         <f>D24*1.25</f>
-        <v>19125</v>
+        <v>18500</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="D25" s="1">
         <f>D24+M$2</f>
-        <v>16250</v>
+        <v>15750</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="D26" s="1">
         <f t="shared" ref="D26:D28" si="8">D25+M$2</f>
-        <v>17200</v>
+        <v>16700</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D27" s="1">
         <f t="shared" si="8"/>
-        <v>18150</v>
+        <v>17650</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="D28" s="1">
         <f t="shared" si="8"/>
-        <v>19100</v>
+        <v>18600</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1864,11 +1864,11 @@
       </c>
       <c r="D29" s="1">
         <f>D28+N$2</f>
-        <v>20050</v>
+        <v>19550</v>
       </c>
       <c r="E29" s="1">
         <f>D29*1.25</f>
-        <v>25062.5</v>
+        <v>24437.5</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="D30" s="1">
         <f t="shared" ref="D30:D33" si="10">D29+N$2</f>
-        <v>21000</v>
+        <v>20500</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="D31" s="1">
         <f t="shared" si="10"/>
-        <v>21950</v>
+        <v>21450</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="D32" s="1">
         <f t="shared" si="10"/>
-        <v>22900</v>
+        <v>22400</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="D33" s="1">
         <f t="shared" si="10"/>
-        <v>23850</v>
+        <v>23350</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1953,11 +1953,11 @@
       </c>
       <c r="D34" s="1">
         <f>D33+O$2</f>
-        <v>24950</v>
+        <v>24450</v>
       </c>
       <c r="E34" s="1">
         <f>D34*1.25</f>
-        <v>31187.5</v>
+        <v>30562.5</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1974,7 +1974,7 @@
       </c>
       <c r="D35" s="1">
         <f t="shared" ref="D35:D38" si="12">D34+O$2</f>
-        <v>26050</v>
+        <v>25550</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="D36" s="1">
         <f t="shared" si="12"/>
-        <v>27150</v>
+        <v>26650</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="D37" s="1">
         <f t="shared" si="12"/>
-        <v>28250</v>
+        <v>27750</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="D38" s="1">
         <f t="shared" si="12"/>
-        <v>29350</v>
+        <v>28850</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -2042,11 +2042,11 @@
       </c>
       <c r="D39" s="1">
         <f>D38+P$2</f>
-        <v>30650</v>
+        <v>30150</v>
       </c>
       <c r="E39" s="1">
         <f>D39*1.25</f>
-        <v>38312.5</v>
+        <v>37687.5</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="D40" s="1">
         <f t="shared" ref="D40:D44" si="14">D39+P$2</f>
-        <v>31950</v>
+        <v>31450</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D41" s="1">
         <f t="shared" si="14"/>
-        <v>33250</v>
+        <v>32750</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="D42" s="1">
         <f t="shared" si="14"/>
-        <v>34550</v>
+        <v>34050</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="D43" s="1">
         <f t="shared" si="14"/>
-        <v>35850</v>
+        <v>35350</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="D44" s="1">
         <f t="shared" si="14"/>
-        <v>37150</v>
+        <v>36650</v>
       </c>
     </row>
   </sheetData>

</xml_diff>